<commit_message>
Sprint 3 day 17
</commit_message>
<xml_diff>
--- a/output/screener_output.xlsx
+++ b/output/screener_output.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L18"/>
+  <dimension ref="A1:O18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -482,6 +482,21 @@
           <t>fcf_yield</t>
         </is>
       </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>sales_cagr_3yr</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>de_declining</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>sales</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -526,6 +541,15 @@
       <c r="L2" t="n">
         <v>0.91</v>
       </c>
+      <c r="M2" t="n">
+        <v>67.58</v>
+      </c>
+      <c r="N2" t="b">
+        <v>0</v>
+      </c>
+      <c r="O2" t="n">
+        <v>68904</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -569,6 +593,15 @@
       </c>
       <c r="L3" t="n">
         <v>0.05</v>
+      </c>
+      <c r="M3" t="n">
+        <v>76.47</v>
+      </c>
+      <c r="N3" t="b">
+        <v>1</v>
+      </c>
+      <c r="O3" t="n">
+        <v>4270</v>
       </c>
     </row>
     <row r="4">
@@ -612,6 +645,15 @@
       <c r="L4" t="n">
         <v>0.78</v>
       </c>
+      <c r="M4" t="n">
+        <v>24.29</v>
+      </c>
+      <c r="N4" t="b">
+        <v>1</v>
+      </c>
+      <c r="O4" t="n">
+        <v>50351</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -656,6 +698,15 @@
       <c r="L5" t="n">
         <v>0.13</v>
       </c>
+      <c r="M5" t="n">
+        <v>42.13</v>
+      </c>
+      <c r="N5" t="b">
+        <v>0</v>
+      </c>
+      <c r="O5" t="n">
+        <v>35517</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -700,6 +751,15 @@
       <c r="L6" t="n">
         <v>8.289999999999999</v>
       </c>
+      <c r="M6" t="n">
+        <v>13.63</v>
+      </c>
+      <c r="N6" t="b">
+        <v>0</v>
+      </c>
+      <c r="O6" t="n">
+        <v>240893</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -744,6 +804,15 @@
       <c r="L7" t="n">
         <v>0.15</v>
       </c>
+      <c r="M7" t="n">
+        <v>68.36</v>
+      </c>
+      <c r="N7" t="b">
+        <v>1</v>
+      </c>
+      <c r="O7" t="n">
+        <v>12375</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -788,6 +857,15 @@
       <c r="L8" t="n">
         <v>0.17</v>
       </c>
+      <c r="M8" t="n">
+        <v>17.8</v>
+      </c>
+      <c r="N8" t="b">
+        <v>0</v>
+      </c>
+      <c r="O8" t="n">
+        <v>35495</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -832,6 +910,15 @@
       <c r="L9" t="n">
         <v>1.22</v>
       </c>
+      <c r="M9" t="n">
+        <v>28.63</v>
+      </c>
+      <c r="N9" t="b">
+        <v>1</v>
+      </c>
+      <c r="O9" t="n">
+        <v>26711</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -876,6 +963,15 @@
       <c r="L10" t="n">
         <v>0.85</v>
       </c>
+      <c r="M10" t="n">
+        <v>13.13</v>
+      </c>
+      <c r="N10" t="b">
+        <v>1</v>
+      </c>
+      <c r="O10" t="n">
+        <v>48497</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -920,6 +1016,15 @@
       <c r="L11" t="n">
         <v>0.59</v>
       </c>
+      <c r="M11" t="n">
+        <v>19.3</v>
+      </c>
+      <c r="N11" t="b">
+        <v>1</v>
+      </c>
+      <c r="O11" t="n">
+        <v>12383</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -964,6 +1069,15 @@
       <c r="L12" t="n">
         <v>3.84</v>
       </c>
+      <c r="M12" t="n">
+        <v>13.4</v>
+      </c>
+      <c r="N12" t="b">
+        <v>0</v>
+      </c>
+      <c r="O12" t="n">
+        <v>109913</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1008,6 +1122,15 @@
       <c r="L13" t="n">
         <v>1.81</v>
       </c>
+      <c r="M13" t="n">
+        <v>15.22</v>
+      </c>
+      <c r="N13" t="b">
+        <v>1</v>
+      </c>
+      <c r="O13" t="n">
+        <v>153670</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1052,6 +1175,15 @@
       <c r="L14" t="n">
         <v>1.43</v>
       </c>
+      <c r="M14" t="n">
+        <v>17.59</v>
+      </c>
+      <c r="N14" t="b">
+        <v>0</v>
+      </c>
+      <c r="O14" t="n">
+        <v>221113</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1096,6 +1228,15 @@
       <c r="L15" t="n">
         <v>0.4</v>
       </c>
+      <c r="M15" t="n">
+        <v>23.78</v>
+      </c>
+      <c r="N15" t="b">
+        <v>0</v>
+      </c>
+      <c r="O15" t="n">
+        <v>16536</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1140,6 +1281,15 @@
       <c r="L16" t="n">
         <v>0.02</v>
       </c>
+      <c r="M16" t="n">
+        <v>13.72</v>
+      </c>
+      <c r="N16" t="b">
+        <v>0</v>
+      </c>
+      <c r="O16" t="n">
+        <v>28011</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1184,6 +1334,15 @@
       <c r="L17" t="n">
         <v>0.33</v>
       </c>
+      <c r="M17" t="n">
+        <v>26.32</v>
+      </c>
+      <c r="N17" t="b">
+        <v>1</v>
+      </c>
+      <c r="O17" t="n">
+        <v>141858</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1227,6 +1386,15 @@
       </c>
       <c r="L18" t="n">
         <v>0.01</v>
+      </c>
+      <c r="M18" t="n">
+        <v>21.14</v>
+      </c>
+      <c r="N18" t="b">
+        <v>0</v>
+      </c>
+      <c r="O18" t="n">
+        <v>18590</v>
       </c>
     </row>
   </sheetData>
@@ -1240,7 +1408,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:O3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1304,6 +1472,21 @@
           <t>fcf_yield</t>
         </is>
       </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>sales_cagr_3yr</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>de_declining</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>sales</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1348,6 +1531,15 @@
       <c r="L2" t="n">
         <v>0.63</v>
       </c>
+      <c r="M2" t="n">
+        <v>19.82</v>
+      </c>
+      <c r="N2" t="b">
+        <v>0</v>
+      </c>
+      <c r="O2" t="n">
+        <v>98692</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1391,6 +1583,15 @@
       </c>
       <c r="L3" t="n">
         <v>-0.27</v>
+      </c>
+      <c r="M3" t="n">
+        <v>23.25</v>
+      </c>
+      <c r="N3" t="b">
+        <v>0</v>
+      </c>
+      <c r="O3" t="n">
+        <v>139078</v>
       </c>
     </row>
   </sheetData>
@@ -1404,7 +1605,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:O10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1468,6 +1669,21 @@
           <t>fcf_yield</t>
         </is>
       </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>sales_cagr_3yr</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>de_declining</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>sales</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1512,6 +1728,15 @@
       <c r="L2" t="n">
         <v>0.91</v>
       </c>
+      <c r="M2" t="n">
+        <v>67.58</v>
+      </c>
+      <c r="N2" t="b">
+        <v>0</v>
+      </c>
+      <c r="O2" t="n">
+        <v>68904</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1556,6 +1781,15 @@
       <c r="L3" t="n">
         <v>0.15</v>
       </c>
+      <c r="M3" t="n">
+        <v>68.36</v>
+      </c>
+      <c r="N3" t="b">
+        <v>1</v>
+      </c>
+      <c r="O3" t="n">
+        <v>12375</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1600,6 +1834,15 @@
       <c r="L4" t="n">
         <v>-4.5</v>
       </c>
+      <c r="M4" t="n">
+        <v>34.6</v>
+      </c>
+      <c r="N4" t="b">
+        <v>0</v>
+      </c>
+      <c r="O4" t="n">
+        <v>96421</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1644,6 +1887,15 @@
       <c r="L5" t="n">
         <v>0.05</v>
       </c>
+      <c r="M5" t="n">
+        <v>76.47</v>
+      </c>
+      <c r="N5" t="b">
+        <v>1</v>
+      </c>
+      <c r="O5" t="n">
+        <v>4270</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1687,6 +1939,15 @@
       </c>
       <c r="L6" t="n">
         <v>0.13</v>
+      </c>
+      <c r="M6" t="n">
+        <v>42.13</v>
+      </c>
+      <c r="N6" t="b">
+        <v>0</v>
+      </c>
+      <c r="O6" t="n">
+        <v>35517</v>
       </c>
     </row>
     <row r="7">
@@ -1730,6 +1991,15 @@
       <c r="L7" t="n">
         <v>0</v>
       </c>
+      <c r="M7" t="n">
+        <v>38.18</v>
+      </c>
+      <c r="N7" t="b">
+        <v>1</v>
+      </c>
+      <c r="O7" t="n">
+        <v>4475</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1774,6 +2044,15 @@
       <c r="L8" t="n">
         <v>0.01</v>
       </c>
+      <c r="M8" t="n">
+        <v>28.13</v>
+      </c>
+      <c r="N8" t="b">
+        <v>1</v>
+      </c>
+      <c r="O8" t="n">
+        <v>50789</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1818,6 +2097,15 @@
       <c r="L9" t="n">
         <v>0.01</v>
       </c>
+      <c r="M9" t="n">
+        <v>9.44</v>
+      </c>
+      <c r="N9" t="b">
+        <v>0</v>
+      </c>
+      <c r="O9" t="n">
+        <v>15206</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1861,6 +2149,15 @@
       </c>
       <c r="L10" t="n">
         <v>0.08</v>
+      </c>
+      <c r="M10" t="n">
+        <v>33.14</v>
+      </c>
+      <c r="N10" t="b">
+        <v>0</v>
+      </c>
+      <c r="O10" t="n">
+        <v>51084</v>
       </c>
     </row>
   </sheetData>
@@ -1874,7 +2171,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L29"/>
+  <dimension ref="A1:O29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1938,6 +2235,21 @@
           <t>fcf_yield</t>
         </is>
       </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>sales_cagr_3yr</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>de_declining</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>sales</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1982,6 +2294,15 @@
       <c r="L2" t="n">
         <v>0.13</v>
       </c>
+      <c r="M2" t="n">
+        <v>42.13</v>
+      </c>
+      <c r="N2" t="b">
+        <v>0</v>
+      </c>
+      <c r="O2" t="n">
+        <v>35517</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2026,6 +2347,15 @@
       <c r="L3" t="n">
         <v>0.4</v>
       </c>
+      <c r="M3" t="n">
+        <v>23.78</v>
+      </c>
+      <c r="N3" t="b">
+        <v>0</v>
+      </c>
+      <c r="O3" t="n">
+        <v>16536</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2069,6 +2399,15 @@
       </c>
       <c r="L4" t="n">
         <v>3</v>
+      </c>
+      <c r="M4" t="n">
+        <v>16.49</v>
+      </c>
+      <c r="N4" t="b">
+        <v>0</v>
+      </c>
+      <c r="O4" t="n">
+        <v>142324</v>
       </c>
     </row>
     <row r="5">
@@ -2112,6 +2451,15 @@
       <c r="L5" t="n">
         <v>0.31</v>
       </c>
+      <c r="M5" t="n">
+        <v>30.19</v>
+      </c>
+      <c r="N5" t="b">
+        <v>0</v>
+      </c>
+      <c r="O5" t="n">
+        <v>283649</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2156,6 +2504,15 @@
       <c r="L6" t="n">
         <v>0.91</v>
       </c>
+      <c r="M6" t="n">
+        <v>67.58</v>
+      </c>
+      <c r="N6" t="b">
+        <v>0</v>
+      </c>
+      <c r="O6" t="n">
+        <v>68904</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2200,6 +2557,15 @@
       <c r="L7" t="n">
         <v>0.04</v>
       </c>
+      <c r="M7" t="n">
+        <v>19.84</v>
+      </c>
+      <c r="N7" t="b">
+        <v>1</v>
+      </c>
+      <c r="O7" t="n">
+        <v>16727</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2244,6 +2610,15 @@
       <c r="L8" t="n">
         <v>10.45</v>
       </c>
+      <c r="M8" t="n">
+        <v>24.46</v>
+      </c>
+      <c r="N8" t="b">
+        <v>1</v>
+      </c>
+      <c r="O8" t="n">
+        <v>899041</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2287,6 +2662,15 @@
       </c>
       <c r="L9" t="n">
         <v>0.85</v>
+      </c>
+      <c r="M9" t="n">
+        <v>13.13</v>
+      </c>
+      <c r="N9" t="b">
+        <v>1</v>
+      </c>
+      <c r="O9" t="n">
+        <v>48497</v>
       </c>
     </row>
     <row r="10">
@@ -2328,6 +2712,13 @@
       <c r="L10" t="n">
         <v>0.18</v>
       </c>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="b">
+        <v>0</v>
+      </c>
+      <c r="O10" t="n">
+        <v>24394</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2370,6 +2761,15 @@
       <c r="L11" t="n">
         <v>2.68</v>
       </c>
+      <c r="M11" t="n">
+        <v>16.3</v>
+      </c>
+      <c r="N11" t="b">
+        <v>0</v>
+      </c>
+      <c r="O11" t="n">
+        <v>110519</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2412,6 +2812,15 @@
       <c r="L12" t="n">
         <v>0.46</v>
       </c>
+      <c r="M12" t="n">
+        <v>6.98</v>
+      </c>
+      <c r="N12" t="b">
+        <v>0</v>
+      </c>
+      <c r="O12" t="n">
+        <v>845966</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2454,6 +2863,15 @@
       <c r="L13" t="n">
         <v>3</v>
       </c>
+      <c r="M13" t="n">
+        <v>20.58</v>
+      </c>
+      <c r="N13" t="b">
+        <v>1</v>
+      </c>
+      <c r="O13" t="n">
+        <v>437928</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2498,6 +2916,15 @@
       <c r="L14" t="n">
         <v>0.99</v>
       </c>
+      <c r="M14" t="n">
+        <v>17.38</v>
+      </c>
+      <c r="N14" t="b">
+        <v>0</v>
+      </c>
+      <c r="O14" t="n">
+        <v>44870</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2541,6 +2968,15 @@
       </c>
       <c r="L15" t="n">
         <v>0.15</v>
+      </c>
+      <c r="M15" t="n">
+        <v>68.36</v>
+      </c>
+      <c r="N15" t="b">
+        <v>1</v>
+      </c>
+      <c r="O15" t="n">
+        <v>12375</v>
       </c>
     </row>
     <row r="16">
@@ -2584,6 +3020,15 @@
       <c r="L16" t="n">
         <v>0.04</v>
       </c>
+      <c r="M16" t="n">
+        <v>18.99</v>
+      </c>
+      <c r="N16" t="b">
+        <v>0</v>
+      </c>
+      <c r="O16" t="n">
+        <v>20487</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2626,6 +3071,15 @@
       <c r="L17" t="n">
         <v>0.95</v>
       </c>
+      <c r="M17" t="n">
+        <v>21.4</v>
+      </c>
+      <c r="N17" t="b">
+        <v>0</v>
+      </c>
+      <c r="O17" t="n">
+        <v>159516</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2669,6 +3123,15 @@
       </c>
       <c r="L18" t="n">
         <v>1.84</v>
+      </c>
+      <c r="M18" t="n">
+        <v>9.06</v>
+      </c>
+      <c r="N18" t="b">
+        <v>0</v>
+      </c>
+      <c r="O18" t="n">
+        <v>12404</v>
       </c>
     </row>
     <row r="19">
@@ -2712,6 +3175,15 @@
       <c r="L19" t="n">
         <v>0.07000000000000001</v>
       </c>
+      <c r="M19" t="n">
+        <v>55.01</v>
+      </c>
+      <c r="N19" t="b">
+        <v>0</v>
+      </c>
+      <c r="O19" t="n">
+        <v>1702</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2756,6 +3228,15 @@
       <c r="L20" t="n">
         <v>0.02</v>
       </c>
+      <c r="M20" t="n">
+        <v>21.75</v>
+      </c>
+      <c r="N20" t="b">
+        <v>0</v>
+      </c>
+      <c r="O20" t="n">
+        <v>19059</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2800,6 +3281,15 @@
       <c r="L21" t="n">
         <v>0.06</v>
       </c>
+      <c r="M21" t="n">
+        <v>14.81</v>
+      </c>
+      <c r="N21" t="b">
+        <v>1</v>
+      </c>
+      <c r="O21" t="n">
+        <v>20521</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2844,6 +3334,15 @@
       <c r="L22" t="n">
         <v>0.08</v>
       </c>
+      <c r="M22" t="n">
+        <v>33.14</v>
+      </c>
+      <c r="N22" t="b">
+        <v>0</v>
+      </c>
+      <c r="O22" t="n">
+        <v>51084</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2887,6 +3386,15 @@
       </c>
       <c r="L23" t="n">
         <v>6.49</v>
+      </c>
+      <c r="M23" t="n">
+        <v>4.97</v>
+      </c>
+      <c r="N23" t="b">
+        <v>1</v>
+      </c>
+      <c r="O23" t="n">
+        <v>45843</v>
       </c>
     </row>
     <row r="24">
@@ -2930,6 +3438,15 @@
       <c r="L24" t="n">
         <v>0.3</v>
       </c>
+      <c r="M24" t="n">
+        <v>19.1</v>
+      </c>
+      <c r="N24" t="b">
+        <v>0</v>
+      </c>
+      <c r="O24" t="n">
+        <v>26645</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2974,6 +3491,15 @@
       <c r="L25" t="n">
         <v>0.07000000000000001</v>
       </c>
+      <c r="M25" t="n">
+        <v>9.91</v>
+      </c>
+      <c r="N25" t="b">
+        <v>0</v>
+      </c>
+      <c r="O25" t="n">
+        <v>30381</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -3018,6 +3544,15 @@
       <c r="L26" t="n">
         <v>0.01</v>
       </c>
+      <c r="M26" t="n">
+        <v>21.14</v>
+      </c>
+      <c r="N26" t="b">
+        <v>0</v>
+      </c>
+      <c r="O26" t="n">
+        <v>18590</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -3062,6 +3597,15 @@
       <c r="L27" t="n">
         <v>0.07000000000000001</v>
       </c>
+      <c r="M27" t="n">
+        <v>5.88</v>
+      </c>
+      <c r="N27" t="b">
+        <v>0</v>
+      </c>
+      <c r="O27" t="n">
+        <v>6427</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -3106,6 +3650,15 @@
       <c r="L28" t="n">
         <v>0.17</v>
       </c>
+      <c r="M28" t="n">
+        <v>17.8</v>
+      </c>
+      <c r="N28" t="b">
+        <v>0</v>
+      </c>
+      <c r="O28" t="n">
+        <v>35495</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -3149,6 +3702,15 @@
       </c>
       <c r="L29" t="n">
         <v>0.63</v>
+      </c>
+      <c r="M29" t="n">
+        <v>19.82</v>
+      </c>
+      <c r="N29" t="b">
+        <v>0</v>
+      </c>
+      <c r="O29" t="n">
+        <v>98692</v>
       </c>
     </row>
   </sheetData>
@@ -3162,7 +3724,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1"/>
+  <dimension ref="A1:O4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3225,6 +3787,180 @@
         <is>
           <t>fcf_yield</t>
         </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>sales_cagr_3yr</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>de_declining</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>sales</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>ITC</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ITC Ltd</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Consumer Staples</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>27.85</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" t="n">
+        <v>15616</v>
+      </c>
+      <c r="G2" t="n">
+        <v>47.85</v>
+      </c>
+      <c r="H2" t="n">
+        <v>4.26</v>
+      </c>
+      <c r="I2" t="n">
+        <v>7.95</v>
+      </c>
+      <c r="J2" t="n">
+        <v>10.08</v>
+      </c>
+      <c r="K2" t="n">
+        <v>65.44</v>
+      </c>
+      <c r="L2" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="M2" t="n">
+        <v>12.89</v>
+      </c>
+      <c r="N2" t="b">
+        <v>1</v>
+      </c>
+      <c r="O2" t="n">
+        <v>70866</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>BOSCHLTD</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Bosch Ltd</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Consumer Discretionary</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>20.64</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" t="n">
+        <v>970</v>
+      </c>
+      <c r="G3" t="n">
+        <v>58.43</v>
+      </c>
+      <c r="H3" t="n">
+        <v>4.23</v>
+      </c>
+      <c r="I3" t="n">
+        <v>6.72</v>
+      </c>
+      <c r="J3" t="n">
+        <v>9.279999999999999</v>
+      </c>
+      <c r="K3" t="n">
+        <v>44.68</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="M3" t="n">
+        <v>19.84</v>
+      </c>
+      <c r="N3" t="b">
+        <v>1</v>
+      </c>
+      <c r="O3" t="n">
+        <v>16727</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>MARUTI</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Maruti Suzuki India Ltd</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Consumer Discretionary</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>15.75</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
+        <v>4936</v>
+      </c>
+      <c r="G4" t="n">
+        <v>20.78</v>
+      </c>
+      <c r="H4" t="n">
+        <v>1.78</v>
+      </c>
+      <c r="I4" t="n">
+        <v>10.51</v>
+      </c>
+      <c r="J4" t="n">
+        <v>12.01</v>
+      </c>
+      <c r="K4" t="n">
+        <v>48.58</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="M4" t="n">
+        <v>26.32</v>
+      </c>
+      <c r="N4" t="b">
+        <v>1</v>
+      </c>
+      <c r="O4" t="n">
+        <v>141858</v>
       </c>
     </row>
   </sheetData>
@@ -3238,7 +3974,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L51"/>
+  <dimension ref="A1:O26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3302,6 +4038,21 @@
           <t>fcf_yield</t>
         </is>
       </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>sales_cagr_3yr</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>de_declining</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>sales</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3346,6 +4097,15 @@
       <c r="L2" t="n">
         <v>0.05</v>
       </c>
+      <c r="M2" t="n">
+        <v>76.47</v>
+      </c>
+      <c r="N2" t="b">
+        <v>1</v>
+      </c>
+      <c r="O2" t="n">
+        <v>4270</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -3390,146 +4150,184 @@
       <c r="L3" t="n">
         <v>0.15</v>
       </c>
+      <c r="M3" t="n">
+        <v>68.36</v>
+      </c>
+      <c r="N3" t="b">
+        <v>1</v>
+      </c>
+      <c r="O3" t="n">
+        <v>12375</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>INDIGO</t>
+          <t>IOC</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Interglobe Aviation Ltd</t>
+          <t>Indian Oil Corporation</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>892.5700000000001</v>
+        <v>23.53</v>
       </c>
       <c r="E4" t="n">
-        <v>0.02</v>
+        <v>0.72</v>
       </c>
       <c r="F4" t="n">
-        <v>9424</v>
+        <v>39635</v>
       </c>
       <c r="G4" t="n">
-        <v>76.23</v>
+        <v>28.61</v>
       </c>
       <c r="H4" t="n">
-        <v>4.27</v>
+        <v>1.25</v>
       </c>
       <c r="I4" t="n">
-        <v>19.31</v>
+        <v>8.01</v>
       </c>
       <c r="J4" t="n">
-        <v>120.69</v>
+        <v>20.1</v>
       </c>
       <c r="K4" t="n">
-        <v>89.68000000000001</v>
+        <v>43.44</v>
       </c>
       <c r="L4" t="n">
-        <v>0.91</v>
+        <v>2.79</v>
+      </c>
+      <c r="M4" t="n">
+        <v>28.73</v>
+      </c>
+      <c r="N4" t="b">
+        <v>1</v>
+      </c>
+      <c r="O4" t="n">
+        <v>776352</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>BAJAJHLDNG</t>
+          <t>ADANIPORTS</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Bajaj Holdings &amp; Investment Ltd</t>
+          <t>Adani Ports &amp; Special Economic Zone Ltd</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>13.58</v>
-      </c>
-      <c r="E5" t="inlineStr"/>
+        <v>15.35</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.9399999999999999</v>
+      </c>
       <c r="F5" t="n">
-        <v>1469</v>
+        <v>8250</v>
       </c>
       <c r="G5" t="n">
-        <v>37.73</v>
+        <v>48.9</v>
       </c>
       <c r="H5" t="n">
-        <v>3.37</v>
+        <v>1.16</v>
       </c>
       <c r="I5" t="n">
-        <v>31.61</v>
+        <v>19.58</v>
       </c>
       <c r="J5" t="n">
-        <v>19.3</v>
+        <v>14.91</v>
       </c>
       <c r="K5" t="n">
-        <v>59.23</v>
+        <v>66.37</v>
       </c>
       <c r="L5" t="n">
-        <v>0.07000000000000001</v>
+        <v>1.22</v>
+      </c>
+      <c r="M5" t="n">
+        <v>28.63</v>
+      </c>
+      <c r="N5" t="b">
+        <v>1</v>
+      </c>
+      <c r="O5" t="n">
+        <v>26711</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>LTIM</t>
+          <t>DMART</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>LTIMindtree Ltd</t>
+          <t>Avenue Supermarts Ltd</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Information Technology</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>22.9</v>
+        <v>13.56</v>
       </c>
       <c r="E6" t="n">
-        <v>0.1</v>
+        <v>0.03</v>
       </c>
       <c r="F6" t="n">
-        <v>1752</v>
+        <v>278</v>
       </c>
       <c r="G6" t="n">
-        <v>64.52</v>
+        <v>72.53</v>
       </c>
       <c r="H6" t="n">
-        <v>4.43</v>
+        <v>1.94</v>
       </c>
       <c r="I6" t="n">
-        <v>30.33</v>
+        <v>20.48</v>
       </c>
       <c r="J6" t="n">
-        <v>24.78</v>
+        <v>22.97</v>
       </c>
       <c r="K6" t="n">
-        <v>69.84</v>
+        <v>48.98</v>
       </c>
       <c r="L6" t="n">
-        <v>0.13</v>
+        <v>0.01</v>
+      </c>
+      <c r="M6" t="n">
+        <v>28.13</v>
+      </c>
+      <c r="N6" t="b">
+        <v>1</v>
+      </c>
+      <c r="O6" t="n">
+        <v>50789</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>TITAN</t>
+          <t>MARUTI</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Titan Company Ltd</t>
+          <t>Maruti Suzuki India Ltd</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -3538,42 +4336,51 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>37.22</v>
+        <v>15.75</v>
       </c>
       <c r="E7" t="n">
-        <v>1.65</v>
+        <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>1506</v>
+        <v>4936</v>
       </c>
       <c r="G7" t="n">
-        <v>10.13</v>
+        <v>20.78</v>
       </c>
       <c r="H7" t="n">
-        <v>3.1</v>
+        <v>1.78</v>
       </c>
       <c r="I7" t="n">
-        <v>20.9</v>
+        <v>10.51</v>
       </c>
       <c r="J7" t="n">
-        <v>20.27</v>
+        <v>12.01</v>
       </c>
       <c r="K7" t="n">
-        <v>67.16</v>
+        <v>48.58</v>
       </c>
       <c r="L7" t="n">
-        <v>0.08</v>
+        <v>0.33</v>
+      </c>
+      <c r="M7" t="n">
+        <v>26.32</v>
+      </c>
+      <c r="N7" t="b">
+        <v>1</v>
+      </c>
+      <c r="O7" t="n">
+        <v>141858</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>GAIL</t>
+          <t>BPCL</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>GAIL (India) Ltd</t>
+          <t>Bharat Petroleum Corporation Ltd</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -3582,84 +4389,104 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>12.86</v>
+        <v>35.51</v>
       </c>
       <c r="E8" t="n">
-        <v>0.28</v>
+        <v>0.72</v>
       </c>
       <c r="F8" t="n">
-        <v>4360</v>
+        <v>25415</v>
       </c>
       <c r="G8" t="n">
-        <v>25.84</v>
+        <v>68.15000000000001</v>
       </c>
       <c r="H8" t="n">
-        <v>0.31</v>
+        <v>1.15</v>
       </c>
       <c r="I8" t="n">
-        <v>11.83</v>
+        <v>8.48</v>
       </c>
       <c r="J8" t="n">
-        <v>8.609999999999999</v>
+        <v>25.79</v>
       </c>
       <c r="K8" t="n">
-        <v>46.19</v>
+        <v>51.97</v>
       </c>
       <c r="L8" t="n">
-        <v>0.28</v>
+        <v>5.42</v>
+      </c>
+      <c r="M8" t="n">
+        <v>24.86</v>
+      </c>
+      <c r="N8" t="b">
+        <v>1</v>
+      </c>
+      <c r="O8" t="n">
+        <v>448083</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>HDFCBANK</t>
+          <t>ONGC</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>HDFC Bank Ltd</t>
+          <t>Oil &amp; Natural Gas Corpn Ltd</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>14.34</v>
-      </c>
-      <c r="E9" t="inlineStr"/>
+        <v>16.94</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.45</v>
+      </c>
       <c r="F9" t="n">
-        <v>2469</v>
+        <v>42060</v>
       </c>
       <c r="G9" t="n">
-        <v>49.42</v>
+        <v>18.15</v>
       </c>
       <c r="H9" t="n">
-        <v>4.33</v>
+        <v>1.11</v>
       </c>
       <c r="I9" t="n">
-        <v>21.95</v>
+        <v>7</v>
       </c>
       <c r="J9" t="n">
-        <v>23.87</v>
+        <v>10.97</v>
       </c>
       <c r="K9" t="n">
-        <v>38.64</v>
+        <v>45.89</v>
       </c>
       <c r="L9" t="n">
-        <v>0.31</v>
+        <v>10.78</v>
+      </c>
+      <c r="M9" t="n">
+        <v>24.86</v>
+      </c>
+      <c r="N9" t="b">
+        <v>1</v>
+      </c>
+      <c r="O9" t="n">
+        <v>591396</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>IOC</t>
+          <t>RELIANCE</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Indian Oil Corporation</t>
+          <t>Reliance Industries Ltd</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -3668,130 +4495,155 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>23.53</v>
+        <v>9.960000000000001</v>
       </c>
       <c r="E10" t="n">
-        <v>0.72</v>
+        <v>0.58</v>
       </c>
       <c r="F10" t="n">
-        <v>39635</v>
+        <v>45207</v>
       </c>
       <c r="G10" t="n">
-        <v>28.61</v>
+        <v>58.34</v>
       </c>
       <c r="H10" t="n">
-        <v>1.25</v>
+        <v>4.21</v>
       </c>
       <c r="I10" t="n">
-        <v>8.01</v>
+        <v>9.609999999999999</v>
       </c>
       <c r="J10" t="n">
-        <v>20.1</v>
+        <v>14.68</v>
       </c>
       <c r="K10" t="n">
-        <v>43.44</v>
+        <v>37.32</v>
       </c>
       <c r="L10" t="n">
-        <v>2.79</v>
+        <v>10.45</v>
+      </c>
+      <c r="M10" t="n">
+        <v>24.46</v>
+      </c>
+      <c r="N10" t="b">
+        <v>1</v>
+      </c>
+      <c r="O10" t="n">
+        <v>899041</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ADANIPORTS</t>
+          <t>ADANIPOWER</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Adani Ports &amp; Special Economic Zone Ltd</t>
+          <t>Adani Power Ltd</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>15.35</v>
+        <v>48.28</v>
       </c>
       <c r="E11" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.8</v>
       </c>
       <c r="F11" t="n">
-        <v>8250</v>
+        <v>10689</v>
       </c>
       <c r="G11" t="n">
-        <v>48.9</v>
+        <v>44.57</v>
       </c>
       <c r="H11" t="n">
-        <v>1.16</v>
+        <v>1.65</v>
       </c>
       <c r="I11" t="n">
-        <v>19.58</v>
-      </c>
-      <c r="J11" t="n">
-        <v>14.91</v>
-      </c>
+        <v>16.09</v>
+      </c>
+      <c r="J11" t="inlineStr"/>
       <c r="K11" t="n">
-        <v>66.37</v>
+        <v>71.45999999999999</v>
       </c>
       <c r="L11" t="n">
-        <v>1.22</v>
+        <v>0.78</v>
+      </c>
+      <c r="M11" t="n">
+        <v>24.29</v>
+      </c>
+      <c r="N11" t="b">
+        <v>1</v>
+      </c>
+      <c r="O11" t="n">
+        <v>50351</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>DMART</t>
+          <t>TATAPOWER</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Avenue Supermarts Ltd</t>
+          <t>Tata Power Company Ltd</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Energy</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>13.56</v>
+        <v>13.23</v>
       </c>
       <c r="E12" t="n">
-        <v>0.03</v>
+        <v>1.66</v>
       </c>
       <c r="F12" t="n">
-        <v>278</v>
+        <v>3569</v>
       </c>
       <c r="G12" t="n">
-        <v>72.53</v>
+        <v>14.5</v>
       </c>
       <c r="H12" t="n">
-        <v>1.94</v>
+        <v>0.49</v>
       </c>
       <c r="I12" t="n">
-        <v>20.48</v>
+        <v>15.51</v>
       </c>
       <c r="J12" t="n">
-        <v>22.97</v>
+        <v>10.43</v>
       </c>
       <c r="K12" t="n">
-        <v>48.98</v>
+        <v>35.78</v>
       </c>
       <c r="L12" t="n">
-        <v>0.01</v>
+        <v>0.22</v>
+      </c>
+      <c r="M12" t="n">
+        <v>23.4</v>
+      </c>
+      <c r="N12" t="b">
+        <v>1</v>
+      </c>
+      <c r="O12" t="n">
+        <v>61449</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>MARUTI</t>
+          <t>TATAMOTORS</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Maruti Suzuki India Ltd</t>
+          <t>Tata Motors Ltd</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -3800,174 +4652,208 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>15.75</v>
+        <v>37.46</v>
       </c>
       <c r="E13" t="n">
-        <v>0</v>
+        <v>1.26</v>
       </c>
       <c r="F13" t="n">
-        <v>4936</v>
+        <v>45133</v>
       </c>
       <c r="G13" t="n">
-        <v>20.78</v>
+        <v>67.06999999999999</v>
       </c>
       <c r="H13" t="n">
-        <v>1.78</v>
+        <v>3.65</v>
       </c>
       <c r="I13" t="n">
-        <v>10.51</v>
-      </c>
-      <c r="J13" t="n">
-        <v>12.01</v>
-      </c>
+        <v>7.72</v>
+      </c>
+      <c r="J13" t="inlineStr"/>
       <c r="K13" t="n">
-        <v>48.58</v>
+        <v>41.56</v>
       </c>
       <c r="L13" t="n">
-        <v>0.33</v>
+        <v>3</v>
+      </c>
+      <c r="M13" t="n">
+        <v>20.58</v>
+      </c>
+      <c r="N13" t="b">
+        <v>1</v>
+      </c>
+      <c r="O13" t="n">
+        <v>437928</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>BPCL</t>
+          <t>BOSCHLTD</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Bharat Petroleum Corporation Ltd</t>
+          <t>Bosch Ltd</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Consumer Discretionary</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>35.51</v>
+        <v>20.64</v>
       </c>
       <c r="E14" t="n">
-        <v>0.72</v>
+        <v>0</v>
       </c>
       <c r="F14" t="n">
-        <v>25415</v>
+        <v>970</v>
       </c>
       <c r="G14" t="n">
-        <v>68.15000000000001</v>
+        <v>58.43</v>
       </c>
       <c r="H14" t="n">
-        <v>1.15</v>
+        <v>4.23</v>
       </c>
       <c r="I14" t="n">
-        <v>8.48</v>
+        <v>6.72</v>
       </c>
       <c r="J14" t="n">
-        <v>25.79</v>
+        <v>9.279999999999999</v>
       </c>
       <c r="K14" t="n">
-        <v>51.97</v>
+        <v>44.68</v>
       </c>
       <c r="L14" t="n">
-        <v>5.42</v>
+        <v>0.04</v>
+      </c>
+      <c r="M14" t="n">
+        <v>19.84</v>
+      </c>
+      <c r="N14" t="b">
+        <v>1</v>
+      </c>
+      <c r="O14" t="n">
+        <v>16727</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ONGC</t>
+          <t>PIDILITIND</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Oil &amp; Natural Gas Corpn Ltd</t>
+          <t>Pidilite Industries Ltd</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Materials</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>16.94</v>
+        <v>20.78</v>
       </c>
       <c r="E15" t="n">
-        <v>0.45</v>
+        <v>0.05</v>
       </c>
       <c r="F15" t="n">
-        <v>42060</v>
+        <v>955</v>
       </c>
       <c r="G15" t="n">
-        <v>18.15</v>
+        <v>36.12</v>
       </c>
       <c r="H15" t="n">
-        <v>1.11</v>
+        <v>1.01</v>
       </c>
       <c r="I15" t="n">
-        <v>7</v>
+        <v>11.84</v>
       </c>
       <c r="J15" t="n">
-        <v>10.97</v>
+        <v>13.49</v>
       </c>
       <c r="K15" t="n">
-        <v>45.89</v>
+        <v>62.19</v>
       </c>
       <c r="L15" t="n">
-        <v>10.78</v>
+        <v>0.59</v>
+      </c>
+      <c r="M15" t="n">
+        <v>19.3</v>
+      </c>
+      <c r="N15" t="b">
+        <v>1</v>
+      </c>
+      <c r="O15" t="n">
+        <v>12383</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>RELIANCE</t>
+          <t>HINDALCO</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Reliance Industries Ltd</t>
+          <t>Hindalco Industries Ltd</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Materials</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>9.960000000000001</v>
+        <v>9.57</v>
       </c>
       <c r="E16" t="n">
-        <v>0.58</v>
+        <v>0.53</v>
       </c>
       <c r="F16" t="n">
-        <v>45207</v>
+        <v>9789</v>
       </c>
       <c r="G16" t="n">
-        <v>58.34</v>
+        <v>56.45</v>
       </c>
       <c r="H16" t="n">
-        <v>4.21</v>
+        <v>0.98</v>
       </c>
       <c r="I16" t="n">
-        <v>9.609999999999999</v>
+        <v>10.59</v>
       </c>
       <c r="J16" t="n">
-        <v>14.68</v>
+        <v>13.07</v>
       </c>
       <c r="K16" t="n">
-        <v>37.32</v>
+        <v>41.64</v>
       </c>
       <c r="L16" t="n">
-        <v>10.45</v>
+        <v>1.36</v>
+      </c>
+      <c r="M16" t="n">
+        <v>17.83</v>
+      </c>
+      <c r="N16" t="b">
+        <v>1</v>
+      </c>
+      <c r="O16" t="n">
+        <v>215962</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ADANIPOWER</t>
+          <t>NTPC</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Adani Power Ltd</t>
+          <t>NTPC Ltd</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -3976,1507 +4862,517 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>48.28</v>
+        <v>13.27</v>
       </c>
       <c r="E17" t="n">
-        <v>0.8</v>
+        <v>1.48</v>
       </c>
       <c r="F17" t="n">
-        <v>10689</v>
+        <v>8644</v>
       </c>
       <c r="G17" t="n">
-        <v>44.57</v>
+        <v>30.8</v>
       </c>
       <c r="H17" t="n">
-        <v>1.65</v>
+        <v>0.06</v>
       </c>
       <c r="I17" t="n">
-        <v>16.09</v>
-      </c>
-      <c r="J17" t="inlineStr"/>
+        <v>12.22</v>
+      </c>
+      <c r="J17" t="n">
+        <v>8.74</v>
+      </c>
       <c r="K17" t="n">
-        <v>71.45999999999999</v>
+        <v>36.31</v>
       </c>
       <c r="L17" t="n">
-        <v>0.78</v>
+        <v>0.95</v>
+      </c>
+      <c r="M17" t="n">
+        <v>16.97</v>
+      </c>
+      <c r="N17" t="b">
+        <v>1</v>
+      </c>
+      <c r="O17" t="n">
+        <v>178501</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>EICHERMOT</t>
+          <t>INFY</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Eicher Motors Ltd</t>
+          <t>Infosys Ltd</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>22.17</v>
+        <v>29.79</v>
       </c>
       <c r="E18" t="n">
-        <v>0.02</v>
+        <v>0.09</v>
       </c>
       <c r="F18" t="n">
-        <v>890</v>
+        <v>20117</v>
       </c>
       <c r="G18" t="n">
-        <v>15.62</v>
+        <v>35.99</v>
       </c>
       <c r="H18" t="n">
-        <v>4.41</v>
+        <v>4.1</v>
       </c>
       <c r="I18" t="n">
-        <v>11.04</v>
+        <v>13.2</v>
       </c>
       <c r="J18" t="n">
-        <v>12.68</v>
+        <v>11.24</v>
       </c>
       <c r="K18" t="n">
-        <v>53.22</v>
+        <v>59.85</v>
       </c>
       <c r="L18" t="n">
-        <v>0.4</v>
+        <v>1.81</v>
+      </c>
+      <c r="M18" t="n">
+        <v>15.22</v>
+      </c>
+      <c r="N18" t="b">
+        <v>1</v>
+      </c>
+      <c r="O18" t="n">
+        <v>153670</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>TATAPOWER</t>
+          <t>SHREECEM</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Tata Power Company Ltd</t>
+          <t>Shree Cement Ltd</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Energy</t>
+          <t>Materials</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>13.23</v>
+        <v>8.369999999999999</v>
       </c>
       <c r="E19" t="n">
-        <v>1.66</v>
+        <v>0.08</v>
       </c>
       <c r="F19" t="n">
-        <v>3569</v>
+        <v>1929</v>
       </c>
       <c r="G19" t="n">
-        <v>14.5</v>
+        <v>25.87</v>
       </c>
       <c r="H19" t="n">
-        <v>0.49</v>
+        <v>3.2</v>
       </c>
       <c r="I19" t="n">
-        <v>15.51</v>
+        <v>10.33</v>
       </c>
       <c r="J19" t="n">
-        <v>10.43</v>
+        <v>11.29</v>
       </c>
       <c r="K19" t="n">
-        <v>35.78</v>
+        <v>43.17</v>
       </c>
       <c r="L19" t="n">
-        <v>0.22</v>
+        <v>0.06</v>
+      </c>
+      <c r="M19" t="n">
+        <v>14.81</v>
+      </c>
+      <c r="N19" t="b">
+        <v>1</v>
+      </c>
+      <c r="O19" t="n">
+        <v>20521</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>APOLLOHOSP</t>
+          <t>BHARTIARTL</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Apollo Hospitals Chain of Indian private hospitals</t>
+          <t>Bharti Airtel Ltd</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Communication Services</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>13.48</v>
+        <v>10.36</v>
       </c>
       <c r="E20" t="n">
-        <v>0.77</v>
+        <v>2.61</v>
       </c>
       <c r="F20" t="n">
-        <v>383</v>
+        <v>27809</v>
       </c>
       <c r="G20" t="n">
-        <v>47.72</v>
+        <v>63.78</v>
       </c>
       <c r="H20" t="n">
-        <v>3.22</v>
+        <v>1.02</v>
       </c>
       <c r="I20" t="n">
-        <v>14.66</v>
+        <v>13.17</v>
       </c>
       <c r="J20" t="n">
-        <v>36.13</v>
+        <v>38.36</v>
       </c>
       <c r="K20" t="n">
-        <v>52.82</v>
+        <v>38.26</v>
       </c>
       <c r="L20" t="n">
-        <v>0.02</v>
+        <v>7.35</v>
+      </c>
+      <c r="M20" t="n">
+        <v>14.23</v>
+      </c>
+      <c r="N20" t="b">
+        <v>1</v>
+      </c>
+      <c r="O20" t="n">
+        <v>149982</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>ICICIBANK</t>
+          <t>SUNPHARMA</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>ICICI Bank Ltd</t>
+          <t>Sun Pharmaceuticals Industries Ltd</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>17.99</v>
-      </c>
-      <c r="E21" t="inlineStr"/>
+        <v>15.09</v>
+      </c>
+      <c r="E21" t="n">
+        <v>0.05</v>
+      </c>
       <c r="F21" t="n">
-        <v>12547</v>
+        <v>11372</v>
       </c>
       <c r="G21" t="n">
-        <v>25.76</v>
+        <v>37.9</v>
       </c>
       <c r="H21" t="n">
-        <v>3.43</v>
+        <v>3.88</v>
       </c>
       <c r="I21" t="n">
-        <v>17.25</v>
+        <v>10.78</v>
       </c>
       <c r="J21" t="n">
-        <v>51.95</v>
+        <v>24.54</v>
       </c>
       <c r="K21" t="n">
-        <v>47.33</v>
+        <v>63.91</v>
       </c>
       <c r="L21" t="n">
-        <v>0.95</v>
+        <v>0.85</v>
+      </c>
+      <c r="M21" t="n">
+        <v>13.13</v>
+      </c>
+      <c r="N21" t="b">
+        <v>1</v>
+      </c>
+      <c r="O21" t="n">
+        <v>48497</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>HAVELLS</t>
+          <t>ITC</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Havells India Ltd</t>
+          <t>ITC Ltd</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Consumer Staples</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>17.07</v>
+        <v>27.85</v>
       </c>
       <c r="E22" t="n">
-        <v>0.04</v>
+        <v>0</v>
       </c>
       <c r="F22" t="n">
-        <v>335</v>
+        <v>15616</v>
       </c>
       <c r="G22" t="n">
-        <v>45.41</v>
+        <v>47.85</v>
       </c>
       <c r="H22" t="n">
-        <v>2.6</v>
+        <v>4.26</v>
       </c>
       <c r="I22" t="n">
-        <v>13.04</v>
+        <v>7.95</v>
       </c>
       <c r="J22" t="n">
-        <v>10.03</v>
+        <v>10.08</v>
       </c>
       <c r="K22" t="n">
-        <v>45.41</v>
+        <v>65.44</v>
       </c>
       <c r="L22" t="n">
-        <v>0.01</v>
+        <v>4.7</v>
+      </c>
+      <c r="M22" t="n">
+        <v>12.89</v>
+      </c>
+      <c r="N22" t="b">
+        <v>1</v>
+      </c>
+      <c r="O22" t="n">
+        <v>70866</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>TATAMOTORS</t>
+          <t>TECHM</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Tata Motors Ltd</t>
+          <t>Tech Mahindra Ltd</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Information Technology</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>37.46</v>
+        <v>8.99</v>
       </c>
       <c r="E23" t="n">
-        <v>1.26</v>
+        <v>0.1</v>
       </c>
       <c r="F23" t="n">
-        <v>45133</v>
+        <v>5058</v>
       </c>
       <c r="G23" t="n">
-        <v>67.06999999999999</v>
+        <v>57.4</v>
       </c>
       <c r="H23" t="n">
-        <v>3.65</v>
+        <v>0.64</v>
       </c>
       <c r="I23" t="n">
-        <v>7.72</v>
-      </c>
-      <c r="J23" t="inlineStr"/>
+        <v>8.4</v>
+      </c>
+      <c r="J23" t="n">
+        <v>-10.99</v>
+      </c>
       <c r="K23" t="n">
-        <v>41.56</v>
+        <v>42.99</v>
       </c>
       <c r="L23" t="n">
-        <v>3</v>
+        <v>0.17</v>
+      </c>
+      <c r="M23" t="n">
+        <v>11.16</v>
+      </c>
+      <c r="N23" t="b">
+        <v>1</v>
+      </c>
+      <c r="O23" t="n">
+        <v>51996</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>BOSCHLTD</t>
+          <t>ABB</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Bosch Ltd</t>
+          <t>Abbott India Ltd</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>20.64</v>
+        <v>32.47</v>
       </c>
       <c r="E24" t="n">
-        <v>0</v>
+        <v>0.02</v>
       </c>
       <c r="F24" t="n">
-        <v>970</v>
+        <v>5622</v>
       </c>
       <c r="G24" t="n">
-        <v>58.43</v>
+        <v>75.58</v>
       </c>
       <c r="H24" t="n">
-        <v>4.23</v>
+        <v>0.96</v>
       </c>
       <c r="I24" t="n">
-        <v>6.72</v>
+        <v>9.720000000000001</v>
       </c>
       <c r="J24" t="n">
-        <v>9.279999999999999</v>
+        <v>21.69</v>
       </c>
       <c r="K24" t="n">
-        <v>44.68</v>
+        <v>73.26000000000001</v>
       </c>
       <c r="L24" t="n">
-        <v>0.04</v>
+        <v>0.37</v>
+      </c>
+      <c r="M24" t="n">
+        <v>10.71</v>
+      </c>
+      <c r="N24" t="b">
+        <v>1</v>
+      </c>
+      <c r="O24" t="n">
+        <v>5849</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>MOTHERSON</t>
+          <t>CIPLA</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Samvardhana Motherson International Ltd</t>
+          <t>Cipla Ltd</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Consumer Discretionary</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>11.55</v>
+        <v>15.55</v>
       </c>
       <c r="E25" t="n">
-        <v>0.76</v>
+        <v>0.02</v>
       </c>
       <c r="F25" t="n">
-        <v>925</v>
+        <v>1152</v>
       </c>
       <c r="G25" t="n">
-        <v>9.539999999999999</v>
+        <v>59.75</v>
       </c>
       <c r="H25" t="n">
-        <v>2.18</v>
+        <v>0.12</v>
       </c>
       <c r="I25" t="n">
-        <v>9.210000000000001</v>
+        <v>9.51</v>
       </c>
       <c r="J25" t="n">
-        <v>7.56</v>
+        <v>22.73</v>
       </c>
       <c r="K25" t="n">
-        <v>32.73</v>
+        <v>62.3</v>
       </c>
       <c r="L25" t="n">
-        <v>0.63</v>
+        <v>0.26</v>
+      </c>
+      <c r="M25" t="n">
+        <v>10.39</v>
+      </c>
+      <c r="N25" t="b">
+        <v>1</v>
+      </c>
+      <c r="O25" t="n">
+        <v>25774</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>KOTAKBANK</t>
+          <t>TORNTPHARM</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Kotak Mahindra Bank Ltd</t>
+          <t>Torrent Pharmaceuticals Ltd</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Financials</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>14.01</v>
-      </c>
-      <c r="E26" t="inlineStr"/>
+        <v>24.15</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0.59</v>
+      </c>
       <c r="F26" t="n">
-        <v>6766</v>
+        <v>3106</v>
       </c>
       <c r="G26" t="n">
-        <v>32.9</v>
+        <v>46.4</v>
       </c>
       <c r="H26" t="n">
-        <v>1.51</v>
+        <v>1.22</v>
       </c>
       <c r="I26" t="n">
-        <v>13.52</v>
+        <v>6.93</v>
       </c>
       <c r="J26" t="n">
-        <v>20.38</v>
+        <v>30.59</v>
       </c>
       <c r="K26" t="n">
-        <v>37.21</v>
+        <v>58.92</v>
       </c>
       <c r="L26" t="n">
-        <v>1.57</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>PIDILITIND</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Pidilite Industries Ltd</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>Materials</t>
-        </is>
-      </c>
-      <c r="D27" t="n">
-        <v>20.78</v>
-      </c>
-      <c r="E27" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="F27" t="n">
-        <v>955</v>
-      </c>
-      <c r="G27" t="n">
-        <v>36.12</v>
-      </c>
-      <c r="H27" t="n">
-        <v>1.01</v>
-      </c>
-      <c r="I27" t="n">
-        <v>11.84</v>
-      </c>
-      <c r="J27" t="n">
-        <v>13.49</v>
-      </c>
-      <c r="K27" t="n">
-        <v>62.19</v>
-      </c>
-      <c r="L27" t="n">
-        <v>0.59</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>IRFC</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Indian Railway Finance Corporation Ltd</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>Financials</t>
-        </is>
-      </c>
-      <c r="D28" t="n">
-        <v>13.04</v>
-      </c>
-      <c r="E28" t="inlineStr"/>
-      <c r="F28" t="n">
-        <v>7906</v>
-      </c>
-      <c r="G28" t="n">
-        <v>9.81</v>
-      </c>
-      <c r="H28" t="n">
-        <v>2.82</v>
-      </c>
-      <c r="I28" t="n">
-        <v>19.07</v>
-      </c>
-      <c r="J28" t="n">
-        <v>23.25</v>
-      </c>
-      <c r="K28" t="n">
-        <v>38.41</v>
-      </c>
-      <c r="L28" t="n">
-        <v>0.3</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>ICICIGI</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>ICICI Lombard General Insurance Company Ltd</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>Financials</t>
-        </is>
-      </c>
-      <c r="D29" t="n">
-        <v>15.72</v>
-      </c>
-      <c r="E29" t="inlineStr"/>
-      <c r="F29" t="n">
-        <v>486</v>
-      </c>
-      <c r="G29" t="n">
-        <v>49</v>
-      </c>
-      <c r="H29" t="n">
-        <v>3.46</v>
-      </c>
-      <c r="I29" t="n">
-        <v>12.91</v>
-      </c>
-      <c r="J29" t="n">
-        <v>12.84</v>
-      </c>
-      <c r="K29" t="n">
-        <v>49.33</v>
-      </c>
-      <c r="L29" t="n">
-        <v>0.04</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>ADANIENSOL</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Adani Energy Solutions Ltd</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>Energy</t>
-        </is>
-      </c>
-      <c r="D30" t="n">
-        <v>9.460000000000001</v>
-      </c>
-      <c r="E30" t="n">
-        <v>2.93</v>
-      </c>
-      <c r="F30" t="n">
-        <v>1095</v>
-      </c>
-      <c r="G30" t="n">
-        <v>58.5</v>
-      </c>
-      <c r="H30" t="n">
-        <v>1.65</v>
-      </c>
-      <c r="I30" t="n">
-        <v>17.85</v>
-      </c>
-      <c r="J30" t="n">
-        <v>16.43</v>
-      </c>
-      <c r="K30" t="n">
-        <v>34.69</v>
-      </c>
-      <c r="L30" t="n">
-        <v>0.31</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>HINDALCO</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>Hindalco Industries Ltd</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>Materials</t>
-        </is>
-      </c>
-      <c r="D31" t="n">
-        <v>9.57</v>
-      </c>
-      <c r="E31" t="n">
-        <v>0.53</v>
-      </c>
-      <c r="F31" t="n">
-        <v>9789</v>
-      </c>
-      <c r="G31" t="n">
-        <v>56.45</v>
-      </c>
-      <c r="H31" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="I31" t="n">
-        <v>10.59</v>
-      </c>
-      <c r="J31" t="n">
-        <v>13.07</v>
-      </c>
-      <c r="K31" t="n">
-        <v>41.64</v>
-      </c>
-      <c r="L31" t="n">
-        <v>1.36</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>ASIANPAINT</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>Asian Paints Indian Multi-National Paint and Coating Manufacturing Company</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>Materials</t>
-        </is>
-      </c>
-      <c r="D32" t="n">
-        <v>29.68</v>
-      </c>
-      <c r="E32" t="n">
-        <v>0.13</v>
-      </c>
-      <c r="F32" t="n">
-        <v>3556</v>
-      </c>
-      <c r="G32" t="n">
-        <v>73.37</v>
-      </c>
-      <c r="H32" t="n">
-        <v>2.42</v>
-      </c>
-      <c r="I32" t="n">
-        <v>13.03</v>
-      </c>
-      <c r="J32" t="n">
-        <v>20.28</v>
-      </c>
-      <c r="K32" t="n">
-        <v>66.59999999999999</v>
-      </c>
-      <c r="L32" t="n">
         <v>0.17</v>
       </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>LT</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>Larsen &amp; Toubro Ltd</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>Industrials</t>
-        </is>
-      </c>
-      <c r="D33" t="n">
-        <v>77.67</v>
-      </c>
-      <c r="E33" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="F33" t="n">
-        <v>16087</v>
-      </c>
-      <c r="G33" t="n">
-        <v>30.8</v>
-      </c>
-      <c r="H33" t="n">
-        <v>1.26</v>
-      </c>
-      <c r="I33" t="n">
-        <v>10.34</v>
-      </c>
-      <c r="J33" t="n">
-        <v>8.76</v>
-      </c>
-      <c r="K33" t="n">
-        <v>57.41</v>
-      </c>
-      <c r="L33" t="n">
-        <v>1.43</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>BAJAJ-AUTO</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>Bajaj Auto Ltd</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>Consumer Discretionary</t>
-        </is>
-      </c>
-      <c r="D34" t="n">
-        <v>26.61</v>
-      </c>
-      <c r="E34" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="F34" t="n">
-        <v>6486</v>
-      </c>
-      <c r="G34" t="n">
-        <v>29.91</v>
-      </c>
-      <c r="H34" t="n">
-        <v>3.59</v>
-      </c>
-      <c r="I34" t="n">
-        <v>8.130000000000001</v>
-      </c>
-      <c r="J34" t="n">
-        <v>9.359999999999999</v>
-      </c>
-      <c r="K34" t="n">
-        <v>62.45</v>
-      </c>
-      <c r="L34" t="n">
-        <v>0.99</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>NTPC</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>NTPC Ltd</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>Energy</t>
-        </is>
-      </c>
-      <c r="D35" t="n">
-        <v>13.27</v>
-      </c>
-      <c r="E35" t="n">
-        <v>1.48</v>
-      </c>
-      <c r="F35" t="n">
-        <v>8644</v>
-      </c>
-      <c r="G35" t="n">
-        <v>30.8</v>
-      </c>
-      <c r="H35" t="n">
-        <v>0.06</v>
-      </c>
-      <c r="I35" t="n">
-        <v>12.22</v>
-      </c>
-      <c r="J35" t="n">
-        <v>8.74</v>
-      </c>
-      <c r="K35" t="n">
-        <v>36.31</v>
-      </c>
-      <c r="L35" t="n">
-        <v>0.95</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>COALINDIA</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>Coal India Ltd</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>Materials</t>
-        </is>
-      </c>
-      <c r="D36" t="n">
-        <v>45.17</v>
-      </c>
-      <c r="E36" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="F36" t="n">
-        <v>13617</v>
-      </c>
-      <c r="G36" t="n">
-        <v>34.27</v>
-      </c>
-      <c r="H36" t="n">
-        <v>4.38</v>
-      </c>
-      <c r="I36" t="n">
-        <v>7.4</v>
-      </c>
-      <c r="J36" t="n">
-        <v>16.43</v>
-      </c>
-      <c r="K36" t="n">
-        <v>69.94</v>
-      </c>
-      <c r="L36" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>SBIN</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>State Bank of India</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>Financials</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr"/>
-      <c r="E37" t="inlineStr"/>
-      <c r="F37" t="n">
-        <v>21632</v>
-      </c>
-      <c r="G37" t="n">
-        <v>54.93</v>
-      </c>
-      <c r="H37" t="n">
-        <v>0.42</v>
-      </c>
-      <c r="I37" t="n">
-        <v>11.63</v>
-      </c>
-      <c r="J37" t="n">
-        <v>83.41</v>
-      </c>
-      <c r="K37" t="n">
-        <v>29.82</v>
-      </c>
-      <c r="L37" t="n">
-        <v>0.9</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>CANBK</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>Canara Bank</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>Financials</t>
-        </is>
-      </c>
-      <c r="D38" t="n">
-        <v>16.72</v>
-      </c>
-      <c r="E38" t="inlineStr"/>
-      <c r="F38" t="n">
-        <v>13296</v>
-      </c>
-      <c r="G38" t="n">
-        <v>36.74</v>
-      </c>
-      <c r="H38" t="n">
-        <v>3.81</v>
-      </c>
-      <c r="I38" t="n">
-        <v>18.18</v>
-      </c>
-      <c r="J38" t="n">
-        <v>85.78</v>
-      </c>
-      <c r="K38" t="n">
-        <v>37.53</v>
-      </c>
-      <c r="L38" t="n">
-        <v>2.68</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>INFY</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>Infosys Ltd</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>Information Technology</t>
-        </is>
-      </c>
-      <c r="D39" t="n">
-        <v>29.79</v>
-      </c>
-      <c r="E39" t="n">
-        <v>0.09</v>
-      </c>
-      <c r="F39" t="n">
-        <v>20117</v>
-      </c>
-      <c r="G39" t="n">
-        <v>35.99</v>
-      </c>
-      <c r="H39" t="n">
-        <v>4.1</v>
-      </c>
-      <c r="I39" t="n">
-        <v>13.2</v>
-      </c>
-      <c r="J39" t="n">
-        <v>11.24</v>
-      </c>
-      <c r="K39" t="n">
-        <v>59.85</v>
-      </c>
-      <c r="L39" t="n">
-        <v>1.81</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>SHREECEM</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>Shree Cement Ltd</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>Materials</t>
-        </is>
-      </c>
-      <c r="D40" t="n">
-        <v>8.369999999999999</v>
-      </c>
-      <c r="E40" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="F40" t="n">
-        <v>1929</v>
-      </c>
-      <c r="G40" t="n">
-        <v>25.87</v>
-      </c>
-      <c r="H40" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="I40" t="n">
-        <v>10.33</v>
-      </c>
-      <c r="J40" t="n">
-        <v>11.29</v>
-      </c>
-      <c r="K40" t="n">
-        <v>43.17</v>
-      </c>
-      <c r="L40" t="n">
-        <v>0.06</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>BHARTIARTL</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>Bharti Airtel Ltd</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>Communication Services</t>
-        </is>
-      </c>
-      <c r="D41" t="n">
-        <v>10.36</v>
-      </c>
-      <c r="E41" t="n">
-        <v>2.61</v>
-      </c>
-      <c r="F41" t="n">
-        <v>27809</v>
-      </c>
-      <c r="G41" t="n">
-        <v>63.78</v>
-      </c>
-      <c r="H41" t="n">
-        <v>1.02</v>
-      </c>
-      <c r="I41" t="n">
-        <v>13.17</v>
-      </c>
-      <c r="J41" t="n">
-        <v>38.36</v>
-      </c>
-      <c r="K41" t="n">
-        <v>38.26</v>
-      </c>
-      <c r="L41" t="n">
-        <v>7.35</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>DRREDDY</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>Dr Reddys Laboratories Ltd</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>Healthcare</t>
-        </is>
-      </c>
-      <c r="D42" t="n">
-        <v>19.74</v>
-      </c>
-      <c r="E42" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="F42" t="n">
-        <v>509</v>
-      </c>
-      <c r="G42" t="n">
-        <v>11.73</v>
-      </c>
-      <c r="H42" t="n">
-        <v>0.09</v>
-      </c>
-      <c r="I42" t="n">
-        <v>12.64</v>
-      </c>
-      <c r="J42" t="n">
-        <v>23.39</v>
-      </c>
-      <c r="K42" t="n">
-        <v>52.36</v>
-      </c>
-      <c r="L42" t="n">
-        <v>0.02</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>TCS</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>Tata Consultancy Services Ltd</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>Information Technology</t>
-        </is>
-      </c>
-      <c r="D43" t="n">
-        <v>50.94</v>
-      </c>
-      <c r="E43" t="n">
-        <v>0.09</v>
-      </c>
-      <c r="F43" t="n">
-        <v>38247</v>
-      </c>
-      <c r="G43" t="n">
-        <v>78.69</v>
-      </c>
-      <c r="H43" t="n">
-        <v>1.62</v>
-      </c>
-      <c r="I43" t="n">
-        <v>10.46</v>
-      </c>
-      <c r="J43" t="n">
-        <v>7.87</v>
-      </c>
-      <c r="K43" t="n">
-        <v>67.95999999999999</v>
-      </c>
-      <c r="L43" t="n">
-        <v>8.289999999999999</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>TATASTEEL</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>Tata Steel Ltd</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>Materials</t>
-        </is>
-      </c>
-      <c r="D44" t="n">
-        <v>-5.33</v>
-      </c>
-      <c r="E44" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="F44" t="n">
-        <v>6048</v>
-      </c>
-      <c r="G44" t="n">
-        <v>48.97</v>
-      </c>
-      <c r="H44" t="n">
+      <c r="M26" t="n">
+        <v>10.25</v>
+      </c>
+      <c r="N26" t="b">
         <v>1</v>
       </c>
-      <c r="I44" t="n">
-        <v>7.77</v>
-      </c>
-      <c r="J44" t="inlineStr"/>
-      <c r="K44" t="n">
-        <v>15.12</v>
-      </c>
-      <c r="L44" t="n">
-        <v>1.64</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>HCLTECH</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>HCL Technologies Ltd</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>Information Technology</t>
-        </is>
-      </c>
-      <c r="D45" t="n">
-        <v>23.01</v>
-      </c>
-      <c r="E45" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="F45" t="n">
-        <v>15840</v>
-      </c>
-      <c r="G45" t="n">
-        <v>63.63</v>
-      </c>
-      <c r="H45" t="n">
-        <v>1.99</v>
-      </c>
-      <c r="I45" t="n">
-        <v>12.71</v>
-      </c>
-      <c r="J45" t="n">
-        <v>9.19</v>
-      </c>
-      <c r="K45" t="n">
-        <v>62.04</v>
-      </c>
-      <c r="L45" t="n">
-        <v>3.84</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>SUNPHARMA</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>Sun Pharmaceuticals Industries Ltd</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>Healthcare</t>
-        </is>
-      </c>
-      <c r="D46" t="n">
-        <v>15.09</v>
-      </c>
-      <c r="E46" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="F46" t="n">
-        <v>11372</v>
-      </c>
-      <c r="G46" t="n">
-        <v>37.9</v>
-      </c>
-      <c r="H46" t="n">
-        <v>3.88</v>
-      </c>
-      <c r="I46" t="n">
-        <v>10.78</v>
-      </c>
-      <c r="J46" t="n">
-        <v>24.54</v>
-      </c>
-      <c r="K46" t="n">
-        <v>63.91</v>
-      </c>
-      <c r="L46" t="n">
-        <v>0.85</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>ITC</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>ITC Ltd</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>Consumer Staples</t>
-        </is>
-      </c>
-      <c r="D47" t="n">
-        <v>27.85</v>
-      </c>
-      <c r="E47" t="n">
-        <v>0</v>
-      </c>
-      <c r="F47" t="n">
-        <v>15616</v>
-      </c>
-      <c r="G47" t="n">
-        <v>47.85</v>
-      </c>
-      <c r="H47" t="n">
-        <v>4.26</v>
-      </c>
-      <c r="I47" t="n">
-        <v>7.95</v>
-      </c>
-      <c r="J47" t="n">
-        <v>10.08</v>
-      </c>
-      <c r="K47" t="n">
-        <v>65.44</v>
-      </c>
-      <c r="L47" t="n">
-        <v>4.7</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>TECHM</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>Tech Mahindra Ltd</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>Information Technology</t>
-        </is>
-      </c>
-      <c r="D48" t="n">
-        <v>8.99</v>
-      </c>
-      <c r="E48" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="F48" t="n">
-        <v>5058</v>
-      </c>
-      <c r="G48" t="n">
-        <v>57.4</v>
-      </c>
-      <c r="H48" t="n">
-        <v>0.64</v>
-      </c>
-      <c r="I48" t="n">
-        <v>8.4</v>
-      </c>
-      <c r="J48" t="n">
-        <v>-10.99</v>
-      </c>
-      <c r="K48" t="n">
-        <v>42.99</v>
-      </c>
-      <c r="L48" t="n">
-        <v>0.17</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>ABB</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>Abbott India Ltd</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>Industrials</t>
-        </is>
-      </c>
-      <c r="D49" t="n">
-        <v>32.47</v>
-      </c>
-      <c r="E49" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="F49" t="n">
-        <v>5622</v>
-      </c>
-      <c r="G49" t="n">
-        <v>75.58</v>
-      </c>
-      <c r="H49" t="n">
-        <v>0.96</v>
-      </c>
-      <c r="I49" t="n">
-        <v>9.720000000000001</v>
-      </c>
-      <c r="J49" t="n">
-        <v>21.69</v>
-      </c>
-      <c r="K49" t="n">
-        <v>73.26000000000001</v>
-      </c>
-      <c r="L49" t="n">
-        <v>0.37</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>CIPLA</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>Cipla Ltd</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>Healthcare</t>
-        </is>
-      </c>
-      <c r="D50" t="n">
-        <v>15.55</v>
-      </c>
-      <c r="E50" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="F50" t="n">
-        <v>1152</v>
-      </c>
-      <c r="G50" t="n">
-        <v>59.75</v>
-      </c>
-      <c r="H50" t="n">
-        <v>0.12</v>
-      </c>
-      <c r="I50" t="n">
-        <v>9.51</v>
-      </c>
-      <c r="J50" t="n">
-        <v>22.73</v>
-      </c>
-      <c r="K50" t="n">
-        <v>62.3</v>
-      </c>
-      <c r="L50" t="n">
-        <v>0.26</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>TORNTPHARM</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>Torrent Pharmaceuticals Ltd</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>Healthcare</t>
-        </is>
-      </c>
-      <c r="D51" t="n">
-        <v>24.15</v>
-      </c>
-      <c r="E51" t="n">
-        <v>0.59</v>
-      </c>
-      <c r="F51" t="n">
-        <v>3106</v>
-      </c>
-      <c r="G51" t="n">
-        <v>46.4</v>
-      </c>
-      <c r="H51" t="n">
-        <v>1.22</v>
-      </c>
-      <c r="I51" t="n">
-        <v>6.93</v>
-      </c>
-      <c r="J51" t="n">
-        <v>30.59</v>
-      </c>
-      <c r="K51" t="n">
-        <v>58.92</v>
-      </c>
-      <c r="L51" t="n">
-        <v>0.17</v>
+      <c r="O26" t="n">
+        <v>10728</v>
       </c>
     </row>
   </sheetData>

</xml_diff>